<commit_message>
Recette : cas C02, E01, E03, F01, F03, G03, G04 réécrits selon le produit (ECARTS n° 77)
- C02 : le site envoie une demande de séjour en brouillon, acompte au comptoir.
- E01 / E03 : la note de chambre passe par le client et son folio ouvert
  unique ; sinon le ticket attend dans « Notes de chambre en attente ».
- F01 / F03 : pas de plafond de crédit ; le mode « Vente à crédit » et la
  sévérité par âge (Récente, En retard, Critique) remplacent le plafond.
- G03 : passage VIP au recalcul quotidien ; G04 : trois conditions VVIP.
- ROADMAP : plus de « plafonds » pour aite_pos_credit.
- Classeur et plan de recette régénérés (146 cas).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EyNqzBSPujF7p28k4eqzEf
</commit_message>
<xml_diff>
--- a/recette/AITE_HOUSE_cahier_de_recette.xlsx
+++ b/recette/AITE_HOUSE_cahier_de_recette.xlsx
@@ -2729,19 +2729,19 @@
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t>Réserver en ligne avec acompte</t>
+          <t>Envoyer une demande de séjour en ligne</t>
         </is>
       </c>
       <c r="G25" s="21" t="inlineStr">
         <is>
           <t>1. Choisir une chambre.
 2. Renseigner les informations client.
-3. Payer l'acompte en ligne.</t>
+3. Envoyer la demande.</t>
         </is>
       </c>
       <c r="H25" s="21" t="inlineStr">
         <is>
-          <t>La réservation est confirmée, le client reçoit sa confirmation, et l'acompte est enregistré.</t>
+          <t>Une réservation en brouillon est créée au nom du client (sans doublon de contact) ; la réception la confirme et encaisse l'acompte au comptoir (pas de paiement en ligne).</t>
         </is>
       </c>
       <c r="I25" s="24" t="inlineStr">
@@ -3699,8 +3699,8 @@
       <c r="G44" s="21" t="inlineStr">
         <is>
           <t>1. Au POS, composer un ticket.
-2. Paiement → Note de chambre.
-3. Sélectionner la chambre occupée.
+2. Sélectionner le client du séjour.
+3. Paiement → Note de chambre.
 4. Valider.</t>
         </is>
       </c>
@@ -3791,22 +3791,23 @@
       </c>
       <c r="E46" s="21" t="inlineStr">
         <is>
-          <t>Aucune chambre occupée</t>
+          <t>Client sans séjour ouvert (ou avec plusieurs)</t>
         </is>
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>Empêcher un report sur une chambre libre</t>
+          <t>Ne jamais reporter au hasard</t>
         </is>
       </c>
       <c r="G46" s="21" t="inlineStr">
         <is>
-          <t>1. Au POS, ouvrir la liste des chambres pour la note de chambre.</t>
+          <t>1. Au POS, régler en Note de chambre un ticket d'un client sans folio ouvert (ou sans client).
+2. Ouvrir Hôtel → Notes de chambre en attente.</t>
         </is>
       </c>
       <c r="H46" s="21" t="inlineStr">
         <is>
-          <t>Seules les chambres réellement occupées sont proposées ; une chambre libre ne peut pas recevoir de report.</t>
+          <t>Le ticket n'est rattaché à aucun folio : il attend dans « Notes de chambre en attente », où la réception choisit le folio.</t>
         </is>
       </c>
       <c r="I46" s="24" t="inlineStr">
@@ -4094,24 +4095,24 @@
       </c>
       <c r="E52" s="21" t="inlineStr">
         <is>
-          <t>Module installé, client créé</t>
+          <t>Module installé</t>
         </is>
       </c>
       <c r="F52" s="23" t="inlineStr">
         <is>
-          <t>Définir un plafond de crédit client</t>
+          <t>Activer la vente à crédit sur un mode de paiement</t>
         </is>
       </c>
       <c r="G52" s="21" t="inlineStr">
         <is>
-          <t>1. Ouvrir la fiche client.
-2. Renseigner le plafond autorisé.
-3. Enregistrer.</t>
+          <t>1. Point de Vente → Configuration → Modes de paiement.
+2. Ouvrir « Ardoise client ».
+3. Vérifier la case « Vente à crédit ».</t>
         </is>
       </c>
       <c r="H52" s="21" t="inlineStr">
         <is>
-          <t>Le plafond est enregistré et visible sur la fiche.</t>
+          <t>Le mode « Ardoise client » existe dès l'installation, case cochée ; seul un mode coché ouvre une ardoise (pas la Note de chambre). Il n'y a pas de plafond de crédit par client.</t>
         </is>
       </c>
       <c r="I52" s="24" t="inlineStr">
@@ -4146,7 +4147,7 @@
       </c>
       <c r="E53" s="21" t="inlineStr">
         <is>
-          <t>Client avec plafond, session de caisse ouverte</t>
+          <t>Client identifié, session de caisse ouverte</t>
         </is>
       </c>
       <c r="F53" s="23" t="inlineStr">
@@ -4199,22 +4200,23 @@
       </c>
       <c r="E54" s="21" t="inlineStr">
         <is>
-          <t>Client dont l'encours atteint le plafond</t>
+          <t>Ardoises d'âges différents</t>
         </is>
       </c>
       <c r="F54" s="23" t="inlineStr">
         <is>
-          <t>Bloquer un crédit au-delà du plafond</t>
+          <t>Repérer les ardoises à relancer</t>
         </is>
       </c>
       <c r="G54" s="21" t="inlineStr">
         <is>
-          <t>1. Tenter un nouveau crédit dépassant le plafond.</t>
+          <t>1. Ouvrir POS Crédit → Ardoises.
+2. Lire la colonne Sévérité et le tableau de bord du crédit.</t>
         </is>
       </c>
       <c r="H54" s="21" t="inlineStr">
         <is>
-          <t>Le système refuse ou alerte explicitement selon le paramétrage ; aucun dépassement silencieux.</t>
+          <t>Chaque ardoise est classée selon son âge (Récente, En retard, Critique ; Réglée une fois soldée) ; les plus anciennes ressortent dans le tableau de bord. La relance se fait à la main.</t>
         </is>
       </c>
       <c r="I54" s="24" t="inlineStr">
@@ -4818,7 +4820,7 @@
       </c>
       <c r="H66" s="21" t="inlineStr">
         <is>
-          <t>Le niveau passe automatiquement à VIP dès le seuil atteint.</t>
+          <t>Le niveau passe à VIP au recalcul quotidien des statuts (tâche planifiée « Fidélité : recalcul des statuts clients »), dès que les seuils de dépenses ET de visites sont atteints.</t>
         </is>
       </c>
       <c r="I66" s="24" t="inlineStr">
@@ -4863,12 +4865,12 @@
       </c>
       <c r="G67" s="21" t="inlineStr">
         <is>
-          <t>1. Franchir le seuil de dépenses et de visites requis.</t>
+          <t>1. Franchir les seuils de dépenses, de visites et de pôles (hébergement, restauration, prestations) requis.</t>
         </is>
       </c>
       <c r="H67" s="21" t="inlineStr">
         <is>
-          <t>Le niveau VVIP n'est attribué que si les deux conditions paramétrées sont remplies.</t>
+          <t>Le niveau VVIP n'est attribué que si les trois conditions paramétrées sont remplies.</t>
         </is>
       </c>
       <c r="I67" s="24" t="inlineStr">

</xml_diff>